<commit_message>
Update locator.xlsx, locator_reader.py 1/10/26
</commit_message>
<xml_diff>
--- a/framework/data/excel/locators.xlsx
+++ b/framework/data/excel/locators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\_DA\DA4\framework\data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF099292-376C-4695-A9C1-EE9A8EB14074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560C8A77-FF36-4C60-AA0F-7173D6D3CB76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="930" yWindow="2520" windowWidth="12450" windowHeight="13185" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>Page</t>
   </si>
@@ -73,6 +73,36 @@
   </si>
   <si>
     <t>errorMessage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search </t>
+  </si>
+  <si>
+    <t>searchBox</t>
+  </si>
+  <si>
+    <t>searchButton</t>
+  </si>
+  <si>
+    <t>noRowsMessage</t>
+  </si>
+  <si>
+    <t>//div[@id='searchBox-wrapper']/div/div/button</t>
+  </si>
+  <si>
+    <t>//div[@id='root']/div/div/div/div[2]/div/div[2]/div/div/span</t>
+  </si>
+  <si>
+    <t>//*[@id="root"]/div/div/div/div[2]/div[1]/div[2]/table/tbody/tr[1]</t>
+  </si>
+  <si>
+    <t>resultTable</t>
+  </si>
+  <si>
+    <t>//*[@id="root"]/div/div/div/div[2]/div[1]/div[2]/table/tbody/tr[1]/td[2]/div/span</t>
+  </si>
+  <si>
+    <t>firstResultTitle</t>
   </si>
 </sst>
 </file>
@@ -431,13 +461,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.28515625" style="1" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="25.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="63.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -525,6 +555,76 @@
         <v>12</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>